<commit_message>
fix(xlsx): add dropdown validation for dict columns and invert showDropDown logic 基本完成
</commit_message>
<xml_diff>
--- a/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/test-imp.xlsx
+++ b/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/test-imp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IdeaProjects\nop-entropy\nop-seago\nop-seago-list\src\test\resources\_vfs\seago\po\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{312602A0-10E1-4459-9444-06755B073080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C92B73B-5685-4975-9FDD-50D12277C97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{392982CA-C4D8-434C-9678-96E43A892558}"/>
+    <workbookView xWindow="9600" yWindow="1030" windowWidth="28800" windowHeight="15370" xr2:uid="{392982CA-C4D8-434C-9678-96E43A892558}"/>
   </bookViews>
   <sheets>
     <sheet name="TestEntity" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
   <si>
     <t>唯一标识</t>
   </si>
@@ -66,6 +66,10 @@
   </si>
   <si>
     <t>PDM</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>A</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -147,23 +151,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -482,51 +480,48 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="3" max="3" width="8.7265625" style="3"/>
-  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1" t="s">
+      <c r="C2" s="3"/>
+      <c r="D2" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3" s="1"/>
+      <c r="A3" s="3"/>
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="1"/>
+      <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="2" t="s">
         <v>10</v>
       </c>
     </row>
@@ -534,13 +529,13 @@
       <c r="A5">
         <v>2</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="2" t="s">
         <v>11</v>
       </c>
     </row>
@@ -548,13 +543,13 @@
       <c r="A6">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D6" s="5" t="s">
+      <c r="C6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(excel): extract common PO Excel operations into shared xlib
</commit_message>
<xml_diff>
--- a/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/test-imp.xlsx
+++ b/nop-seago/nop-seago-list/src/test/resources/_vfs/seago/po/test-imp.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\IdeaProjects\nop-entropy\nop-seago\nop-seago-list\src\test\resources\_vfs\seago\po\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C92B73B-5685-4975-9FDD-50D12277C97D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA38624D-2719-45FB-8C69-9B722DD032B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9600" yWindow="1030" windowWidth="28800" windowHeight="15370" xr2:uid="{392982CA-C4D8-434C-9678-96E43A892558}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{392982CA-C4D8-434C-9678-96E43A892558}"/>
   </bookViews>
   <sheets>
     <sheet name="TestEntity" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t>唯一标识</t>
   </si>
@@ -66,10 +66,6 @@
   </si>
   <si>
     <t>PDM</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>A</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -547,7 +543,7 @@
         <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>10</v>

</xml_diff>